<commit_message>
impr extension binding (#57) 4cf306db6c7f029d735dd8d648b18d9a90a928b6
</commit_message>
<xml_diff>
--- a/ig/main/StructureDefinition-mesures-number-of-days.xlsx
+++ b/ig/main/StructureDefinition-mesures-number-of-days.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="70">
   <si>
     <t>Property</t>
   </si>
@@ -54,7 +54,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-07-18T09:34:12+00:00</t>
+    <t>2023-07-18T09:34:49+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -223,6 +223,12 @@
   </si>
   <si>
     <t>Value of extension - must be one of a constrained set of the data types (see [Extensibility](http://hl7.org/fhir/R4/extensibility.html) for a list).</t>
+  </si>
+  <si>
+    <t>required</t>
+  </si>
+  <si>
+    <t>https://mos.esante.gouv.fr/NOS/JDV_J164-GlucoseNumberOfDays-ENS/FHIR/JDV-J164-GlucoseNumberOfDays-ENS</t>
   </si>
   <si>
     <t xml:space="preserve">ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
@@ -548,9 +554,9 @@
     <col min="21" max="21" width="1.04296875" customWidth="true" bestFit="true"/>
     <col min="22" max="22" width="1.04296875" customWidth="true" bestFit="true"/>
     <col min="23" max="23" width="1.04296875" customWidth="true" bestFit="true"/>
-    <col min="24" max="24" width="1.04296875" customWidth="true" bestFit="true"/>
+    <col min="24" max="24" width="8.8046875" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="1.04296875" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="1.04296875" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="104.83984375" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="1.04296875" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="10.26171875" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="42.03515625" customWidth="true" bestFit="true"/>
@@ -1040,13 +1046,11 @@
         <v>36</v>
       </c>
       <c r="X5" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="Y5" t="s" s="2">
-        <v>36</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="Y5" s="2"/>
       <c r="Z5" t="s" s="2">
-        <v>36</v>
+        <v>68</v>
       </c>
       <c r="AA5" t="s" s="2">
         <v>36</v>
@@ -1076,7 +1080,7 @@
         <v>41</v>
       </c>
       <c r="AJ5" t="s" s="2">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="AK5" t="s" s="2">
         <v>62</v>

</xml_diff>